<commit_message>
Build the drainage minimum-slope check (Phase 2 sub-check #2)
Same sizing-summary-Excel-vs-reference-table mechanism as velocity, code
basis IPC Table 704.1 (min grade by pipe diameter, mirroring the same
source already used for the Drainage(gravity) velocity minimum). New
DrainageSlopeLimits.xlsx reference table, a Slope sheet on SizingSummary.xlsx,
checks/code_compliance_slope.py, and --slope-excel/--slope-limits-excel CLI
flags writing into the shared CodeCompliance sheet. Pipe-diameter parsing
extracted into checks/sizing_parsing.py, shared with velocity_check. 12 new
tests (70 total). Smoke-tested against the template's sample row and a real
CLI run; a real F12-04-233 acceptance test is blocked on confirming the
drainage plan's actual drawing scale (no dimension entities or $INSUNITS to
calibrate against) -- documented as a follow-up, not faked.
</commit_message>
<xml_diff>
--- a/docs/excel_templates/SizingSummary.xlsx
+++ b/docs/excel_templates/SizingSummary.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Velocity" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Slope" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -532,7 +533,6 @@
           <t>DN50</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -558,7 +558,78 @@
           <t>DN150</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Installed Size</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Upstream Invert (m)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Downstream Invert (m)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Run Length (m)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MH-01 to MH-02</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>150mm</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>981.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>980.95</v>
+      </c>
+      <c r="E2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Sample row, sanity-checked at 1.83% (&gt;=1.04% min for this diameter).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Build and pass the equipment-sizing-vs-calc check (Phase 2 sub-check #3)
Direct calc-vs-drawing comparison, no code-basis reference table needed:
a Required (Calc) vs Installed (Drawing) value per tagged parameter, with
an optional tolerance to absorb legitimate schedule-rounding noise. New
EquipmentSizing sheet on SizingSummary.xlsx, checks/code_compliance_
equipment_sizing.py, and a standalone --equipment-sizing-excel CLI flag.
9 new tests (79 total).

Passed a real F12-04-233 acceptance test with no scale-calibration caveats
(every value came from text extraction, not measured geometry): 1 genuine
FAIL (IRRP-01 undersized vs its own calc), 7 clean passes including the
SP-02/HWP-01/WT-01 real-data edge cases noted in docs/PROCEDURE.md #19.
</commit_message>
<xml_diff>
--- a/docs/excel_templates/SizingSummary.xlsx
+++ b/docs/excel_templates/SizingSummary.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Velocity" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Slope" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EquipmentSizing" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -634,4 +635,86 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Required (Calc)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Installed (Drawing)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Tolerance (%)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SP-02</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Flow (L/s)</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>L/s</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Sample row using a real project's own numbers (F12-04-233, docs/PROCEDURE.md #17/#18): calc sheet requires 0.06 L/s, the P0801 pumps schedule shows 0.30 L/s installed -- passes here since installed exceeds required, but the 5x gap between the two sources is itself worth a human look.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Build and pass the manhole/inspection-chamber sizing check (Phase 2 sub-check #4)
Code basis: UK Approved Document H Table 11 (minimum chamber size by
depth), the best-fitting real standard for private on-site building
drainage -- IPC governs manhole spacing not size, and the US Ten States
Standards' flat 1200mm minimum is a public-sewer rule that doesn't apply
here. Real F12-04-233 manhole schedule data (MH SIZE/APPROXIMATE DEPTH
columns, no drawing-geometry calibration needed) passes cleanly against
the new reference table, matching the velocity+slope baseline exactly
with zero regression.

4 of 5 Phase 2 sub-checks now built and acceptance-tested.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel_templates/SizingSummary.xlsx
+++ b/docs/excel_templates/SizingSummary.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Velocity" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Slope" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="EquipmentSizing" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Manholes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -717,4 +718,60 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tag</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>MH Size (mm)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Approx Depth (m)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MH-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>600X600</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sample row using a real project's own numbers (F12-04-233, docs/PROCEDURE.md #22): P0801 SEWAGE MANHOLES SCHEDULE, square inspection chamber. At 0.6m depth this matches the 0-0.6m tier (min side 100mm) -- 600mm passes comfortably.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>